<commit_message>
Copy-edits to documents (protocol, Word version of questionnaires, and interim report)
</commit_message>
<xml_diff>
--- a/Protocols/End-process - PPS sampling template - example for training.xlsx
+++ b/Protocols/End-process - PPS sampling template - example for training.xlsx
@@ -7653,8 +7653,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BF11AF2F54683D48B47D51E7C5C20D0A" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="739c6c93e1fa3242103328fd7c6fd4fe">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7a2ce8f2-2204-4367-a41c-b735e7c03037" xmlns:ns3="f53cdae7-58e9-463a-80c4-ff1f1a52caeb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="23a554fc1540e055b3dda9e0febfb003" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BF11AF2F54683D48B47D51E7C5C20D0A" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c3ec6b3112fff6afcb2e1bceac7318f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7a2ce8f2-2204-4367-a41c-b735e7c03037" xmlns:ns3="f53cdae7-58e9-463a-80c4-ff1f1a52caeb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1733b412cddd9f821d661af390973bad" ns2:_="" ns3:_="">
     <xsd:import namespace="7a2ce8f2-2204-4367-a41c-b735e7c03037"/>
     <xsd:import namespace="f53cdae7-58e9-463a-80c4-ff1f1a52caeb"/>
     <xsd:element name="properties">
@@ -7947,5 +7947,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D133407F-4B90-4ECC-B7FD-F14E6E6A8F54}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2E441CF-3FA8-4581-9146-776D96C8D146}"/>
 </file>
</xml_diff>